<commit_message>
questionable rule changes - NEEDS CHECKING
</commit_message>
<xml_diff>
--- a/rules/CORE-000238/positive/01/data/unit-test-coreid-CG0147-positive 1.xlsx
+++ b/rules/CORE-000238/positive/01/data/unit-test-coreid-CG0147-positive 1.xlsx
@@ -562,7 +562,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Z5"/>
+  <dimension ref="A1:Z6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1146,6 +1146,116 @@
         </is>
       </c>
       <c r="Z5" s="4" t="inlineStr">
+        <is>
+          <t>USA</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>CDISCPILOT01</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>DM</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>GUARD-RFXEN-OK</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>1115</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>2012-11-30</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>2013-01-23</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>2014-01-01</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>2014-01-20</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>2012-11-23</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>2013-05-20</t>
+        </is>
+      </c>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>701</t>
+        </is>
+      </c>
+      <c r="N6" t="inlineStr">
+        <is>
+          <t>1928</t>
+        </is>
+      </c>
+      <c r="O6" t="n">
+        <v>84</v>
+      </c>
+      <c r="P6" t="inlineStr">
+        <is>
+          <t>YEARS</t>
+        </is>
+      </c>
+      <c r="Q6" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="R6" t="inlineStr">
+        <is>
+          <t>WHITE</t>
+        </is>
+      </c>
+      <c r="S6" t="inlineStr">
+        <is>
+          <t>NOT HISPANIC OR LATINO</t>
+        </is>
+      </c>
+      <c r="T6" t="inlineStr">
+        <is>
+          <t>ZAN_LOW</t>
+        </is>
+      </c>
+      <c r="U6" t="inlineStr">
+        <is>
+          <t>Zanomaline Low Dose (54 mg)</t>
+        </is>
+      </c>
+      <c r="V6" t="inlineStr">
+        <is>
+          <t>ZAN_LOW</t>
+        </is>
+      </c>
+      <c r="W6" t="inlineStr">
+        <is>
+          <t>Zanomaline Low Dose (54 mg)</t>
+        </is>
+      </c>
+      <c r="Z6" t="inlineStr">
         <is>
           <t>USA</t>
         </is>
@@ -1162,7 +1272,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q59"/>
+  <dimension ref="A1:Q61"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5824,6 +5934,164 @@
         <v>55</v>
       </c>
     </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>CDISCPILOT01</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>EX</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>GUARD-RFXEN-OK</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>DEV0001</t>
+        </is>
+      </c>
+      <c r="E60" t="n">
+        <v>1</v>
+      </c>
+      <c r="F60" t="inlineStr">
+        <is>
+          <t>ZANOMALINE</t>
+        </is>
+      </c>
+      <c r="G60" t="n">
+        <v>54</v>
+      </c>
+      <c r="H60" t="inlineStr">
+        <is>
+          <t>mg</t>
+        </is>
+      </c>
+      <c r="I60" t="inlineStr">
+        <is>
+          <t>INJECTION</t>
+        </is>
+      </c>
+      <c r="J60" t="inlineStr">
+        <is>
+          <t>QD</t>
+        </is>
+      </c>
+      <c r="K60" t="inlineStr">
+        <is>
+          <t>SUBCUTANEOUS</t>
+        </is>
+      </c>
+      <c r="L60" t="inlineStr">
+        <is>
+          <t>SDS580-359</t>
+        </is>
+      </c>
+      <c r="M60" t="inlineStr">
+        <is>
+          <t>TREATMENT</t>
+        </is>
+      </c>
+      <c r="N60" t="inlineStr">
+        <is>
+          <t>2014-01-01</t>
+        </is>
+      </c>
+      <c r="O60" t="inlineStr">
+        <is>
+          <t>2014-01-05</t>
+        </is>
+      </c>
+      <c r="P60" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q60" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>CDISCPILOT01</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>EX</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>GUARD-RFXEN-OK</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>DEV0001</t>
+        </is>
+      </c>
+      <c r="E61" t="n">
+        <v>2</v>
+      </c>
+      <c r="F61" t="inlineStr">
+        <is>
+          <t>ZANOMALINE</t>
+        </is>
+      </c>
+      <c r="G61" t="n">
+        <v>54</v>
+      </c>
+      <c r="H61" t="inlineStr">
+        <is>
+          <t>mg</t>
+        </is>
+      </c>
+      <c r="I61" t="inlineStr">
+        <is>
+          <t>INJECTION</t>
+        </is>
+      </c>
+      <c r="J61" t="inlineStr">
+        <is>
+          <t>QD</t>
+        </is>
+      </c>
+      <c r="K61" t="inlineStr">
+        <is>
+          <t>SUBCUTANEOUS</t>
+        </is>
+      </c>
+      <c r="L61" t="inlineStr">
+        <is>
+          <t>SDS580-359</t>
+        </is>
+      </c>
+      <c r="M61" t="inlineStr">
+        <is>
+          <t>TREATMENT</t>
+        </is>
+      </c>
+      <c r="N61" t="inlineStr">
+        <is>
+          <t>2014-01-10</t>
+        </is>
+      </c>
+      <c r="O61" t="inlineStr">
+        <is>
+          <t>2014-01-20</t>
+        </is>
+      </c>
+      <c r="P61" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q61" t="n">
+        <v>1</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>